<commit_message>
data: activate SRC-13 as authority pending (DEC-15)
Workbook: parse check set to validated by manual review, lifecycle set to Authority pending.
Manifest: validated_extraction enabled. Reviewer Raphael Ribot, 2026-10-13 to 14.
Not BPL-confirmed: OD-01 and DEC-08 remain pending BPL.
</commit_message>
<xml_diff>
--- a/packages/orchestrator/sample_corpus/AskBPL_Source_Inventory_v0_1.xlsx
+++ b/packages/orchestrator/sample_corpus/AskBPL_Source_Inventory_v0_1.xlsx
@@ -1,21 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/AskBPL/packages/orchestrator/sample_corpus/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AC1706-041A-3F42-A12F-3AC0B58336D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="29640" windowHeight="23420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Source Inventory" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Counts (ING-13)" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Source Inventory" sheetId="1" r:id="rId1"/>
+    <sheet name="Counts (ING-13)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Source Inventory'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Inventory'!$A$1:$N$31</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -24,460 +40,454 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="148">
-  <si>
-    <t xml:space="preserve">Source ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">File name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chars per page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parse check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In current pilot index</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lifecycle status (ING-9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocking decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes (PRD v1.2 s19.3 / 19.4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner (D-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policy number / dates (from document, to confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewer / date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01 - Emergency Response Procedure (10.02).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pass: text layer present (not yet content-validated)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Procedure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authority pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-03; OD-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2002 document. Check escalation steps, phone numbers, applicability, supersession. Never present as current emergency direction (SAF-8).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01 - Policy for Policy Management.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policy (governance)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">April 2026 document describing the BPL approval process. Used to judge authority of other sources (19.2).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01 - Technology Use (6.13).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-13; OD-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number 'IV. Public 1', describes public-computer rules, application line says All Staff. Different document from HR12, not a version of it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01 - Use of Personal Vehicles (10.95).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1995. Do not repeat an old reimbursement rate as current.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02 - Materials Selection Policy (04.05) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 1. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02 - Policy on Unattended Children (09.05).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 2. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02a - Emergency System-wide Closing Procedure (STAFF) (10.02).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2002 document. Check escalation steps, numbers, applicability, supersession (SAF-8).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02d - Collection Maintenance Procedures (updated 2026).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Updated 2026. Verify applicability and evidence passages. Keep distinct from Materials Selection policy (ING-10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03 - Internal Communications Policy and Norms (10.24) (2).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024. Review confidentiality and current process.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04 - Annual Leave Policy (01.06).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 3. May apply only to non-union staff (19.4). Never compute current entitlements from outdated text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04 - Promotional and Marketing Materials (05.20) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not flagged in 19.3. Confirm status and owner.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05 - Anti Harassment Policy (Revised 10.18) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check dates, eligibility, labor agreements, legal and HR authority.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06 - Conflict of Interest (06.14) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAIL: scanned or image-only (text far below normal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authority pending; extraction blocked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-01; extraction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 4. PDF pages are scanned images; text layer holds almost nothing. Needs validated extraction or manual verification before any indexing (ING-3, ING-11, GATE-04).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06 - Fundraising Policy (12.01).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 5. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07 - Media Relations and Publicity Policy (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07 - Volunteer Manual (12.08).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client test script group 6. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09 - Dress Code Policy (06.06).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 - Whistle Blowers Protection-09.2006 (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11 - Photograhy and Video Policy_Mar2024 (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11554 CP Update to BPL Rules_deck 0423.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design deck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">April 2026 public-rules design deck. Not an approved policy (ING-10, 19.3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 - Custodianship of Library Materials (02.08) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2008. Verify applicability and evidence passages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 - Technology Usage Policy (06.06) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HR12, issued October 2006; applies to all employees, consultants, contractors, temporaries, vendors. Different document from 'Technology Use' (6.13). Check generic 'Company' wording and system references.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 - Crisis Management Policy.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2008. Check escalation instructions, numbers, applicability, supersession (SAF-8).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 - Progressive Discipline Policy (06.06).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check dates, eligibility, labor agreements, legal and HR authority. No disciplinary decisions (GRD-10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 - Service Rating Manual (07.74).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1974 reference. Check current relevance and employee agreement implications.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 - Family and Medical Leave Act  (06.06).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2006. Check dates, eligibility, legal and HR authority. Never calculate current legal entitlements from it (19.4).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 - Social Media Policy (03.22) (1).pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022. Review confidentiality and current process.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ask_BPL_AI_Policy_Test_Script.docx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOCX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Text extracted (Word file)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluation material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excluded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None (not a policy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The 30-question BPL test script (24 in-scope, 6 boundary). Used for GATE-08; never indexed. Counted separately (19.1).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guidelines for Public Behavior Violations.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supporting guidance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 guidance. Supports, and cannot override, the Public Behavior policy (ING-10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SRC-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public Behavior in the Library Policy (updated Jan-26).docx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policy (draft indicators)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OD-02; OD-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filename says updated Jan-26; internal text says 'Issued: June 2026 (TBD)'. Resolve before answering public-behavior questions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How it is computed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Files received</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All rows (AC-1, GATE-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unique by content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHA-256 compared across all 30 files on 2026-10-10; no duplicate content (entered as =B2 because that check was run outside the workbook)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BPL documents (excluding test script)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Policies, procedures, guidance and deck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eligible (BPL-confirmed current)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zero until BPL confirms authority (OD-01)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Includes the extraction-blocked file</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extraction blocked (parse check failed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ING-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excluded from corpus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluation script</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Currently in the pilot index (not confirmed eligible)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Byte-identical to the supplied copies; authority still unconfirmed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indexed AND eligible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cannot be claimed yet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documents with a named open decision (OD-02/03/13)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public behavior, emergency/crisis, technology pair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legend: yellow cells on 'Source Inventory' (Owner, Policy number/dates, Reviewer/date) are for Bath Bilissalou / BPL to fill. Every status above is a team disposition, not BPL approval. Parse check only proves text exists; content validation (GATE-04) is still to do.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="147">
+  <si>
+    <t>Source ID</t>
+  </si>
+  <si>
+    <t>File name</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>Pages</t>
+  </si>
+  <si>
+    <t>Chars per page</t>
+  </si>
+  <si>
+    <t>Parse check</t>
+  </si>
+  <si>
+    <t>In current pilot index</t>
+  </si>
+  <si>
+    <t>Source type</t>
+  </si>
+  <si>
+    <t>Lifecycle status (ING-9)</t>
+  </si>
+  <si>
+    <t>Blocking decision</t>
+  </si>
+  <si>
+    <t>Notes (PRD v1.2 s19.3 / 19.4)</t>
+  </si>
+  <si>
+    <t>Owner (D-02)</t>
+  </si>
+  <si>
+    <t>Policy number / dates (from document, to confirm)</t>
+  </si>
+  <si>
+    <t>Reviewer / date</t>
+  </si>
+  <si>
+    <t>SRC-01</t>
+  </si>
+  <si>
+    <t>01 - Emergency Response Procedure (10.02).pdf</t>
+  </si>
+  <si>
+    <t>PDF</t>
+  </si>
+  <si>
+    <t>Pass: text layer present (not yet content-validated)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Procedure</t>
+  </si>
+  <si>
+    <t>Authority pending</t>
+  </si>
+  <si>
+    <t>OD-03; OD-01</t>
+  </si>
+  <si>
+    <t>2002 document. Check escalation steps, phone numbers, applicability, supersession. Never present as current emergency direction (SAF-8).</t>
+  </si>
+  <si>
+    <t>SRC-02</t>
+  </si>
+  <si>
+    <t>01 - Policy for Policy Management.pdf</t>
+  </si>
+  <si>
+    <t>Policy (governance)</t>
+  </si>
+  <si>
+    <t>OD-01</t>
+  </si>
+  <si>
+    <t>April 2026 document describing the BPL approval process. Used to judge authority of other sources (19.2).</t>
+  </si>
+  <si>
+    <t>SRC-03</t>
+  </si>
+  <si>
+    <t>01 - Technology Use (6.13).pdf</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Policy</t>
+  </si>
+  <si>
+    <t>OD-13; OD-01</t>
+  </si>
+  <si>
+    <t>Number 'IV. Public 1', describes public-computer rules, application line says All Staff. Different document from HR12, not a version of it.</t>
+  </si>
+  <si>
+    <t>SRC-04</t>
+  </si>
+  <si>
+    <t>01 - Use of Personal Vehicles (10.95).pdf</t>
+  </si>
+  <si>
+    <t>1995. Do not repeat an old reimbursement rate as current.</t>
+  </si>
+  <si>
+    <t>SRC-05</t>
+  </si>
+  <si>
+    <t>02 - Materials Selection Policy (04.05) (1).pdf</t>
+  </si>
+  <si>
+    <t>Client test script group 1. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-06</t>
+  </si>
+  <si>
+    <t>02 - Policy on Unattended Children (09.05).pdf</t>
+  </si>
+  <si>
+    <t>Client test script group 2. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-07</t>
+  </si>
+  <si>
+    <t>02a - Emergency System-wide Closing Procedure (STAFF) (10.02).pdf</t>
+  </si>
+  <si>
+    <t>2002 document. Check escalation steps, numbers, applicability, supersession (SAF-8).</t>
+  </si>
+  <si>
+    <t>SRC-08</t>
+  </si>
+  <si>
+    <t>02d - Collection Maintenance Procedures (updated 2026).pdf</t>
+  </si>
+  <si>
+    <t>Updated 2026. Verify applicability and evidence passages. Keep distinct from Materials Selection policy (ING-10).</t>
+  </si>
+  <si>
+    <t>SRC-09</t>
+  </si>
+  <si>
+    <t>03 - Internal Communications Policy and Norms (10.24) (2).pdf</t>
+  </si>
+  <si>
+    <t>2024. Review confidentiality and current process.</t>
+  </si>
+  <si>
+    <t>SRC-10</t>
+  </si>
+  <si>
+    <t>04 - Annual Leave Policy (01.06).pdf</t>
+  </si>
+  <si>
+    <t>Client test script group 3. May apply only to non-union staff (19.4). Never compute current entitlements from outdated text.</t>
+  </si>
+  <si>
+    <t>SRC-11</t>
+  </si>
+  <si>
+    <t>04 - Promotional and Marketing Materials (05.20) (1).pdf</t>
+  </si>
+  <si>
+    <t>Not flagged in 19.3. Confirm status and owner.</t>
+  </si>
+  <si>
+    <t>SRC-12</t>
+  </si>
+  <si>
+    <t>05 - Anti Harassment Policy (Revised 10.18) (1).pdf</t>
+  </si>
+  <si>
+    <t>Check dates, eligibility, labor agreements, legal and HR authority.</t>
+  </si>
+  <si>
+    <t>SRC-13</t>
+  </si>
+  <si>
+    <t>06 - Conflict of Interest (06.14) (1).pdf</t>
+  </si>
+  <si>
+    <t>OD-01; extraction</t>
+  </si>
+  <si>
+    <t>Client test script group 4. PDF pages are scanned images; text layer holds almost nothing. Needs validated extraction or manual verification before any indexing (ING-3, ING-11, GATE-04).</t>
+  </si>
+  <si>
+    <t>SRC-14</t>
+  </si>
+  <si>
+    <t>06 - Fundraising Policy (12.01).pdf</t>
+  </si>
+  <si>
+    <t>Client test script group 5. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-15</t>
+  </si>
+  <si>
+    <t>07 - Media Relations and Publicity Policy (1).pdf</t>
+  </si>
+  <si>
+    <t>SRC-16</t>
+  </si>
+  <si>
+    <t>07 - Volunteer Manual (12.08).pdf</t>
+  </si>
+  <si>
+    <t>Client test script group 6. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-17</t>
+  </si>
+  <si>
+    <t>09 - Dress Code Policy (06.06).pdf</t>
+  </si>
+  <si>
+    <t>SRC-18</t>
+  </si>
+  <si>
+    <t>10 - Whistle Blowers Protection-09.2006 (1).pdf</t>
+  </si>
+  <si>
+    <t>SRC-19</t>
+  </si>
+  <si>
+    <t>11 - Photograhy and Video Policy_Mar2024 (1).pdf</t>
+  </si>
+  <si>
+    <t>2024. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-20</t>
+  </si>
+  <si>
+    <t>11554 CP Update to BPL Rules_deck 0423.pdf</t>
+  </si>
+  <si>
+    <t>Design deck</t>
+  </si>
+  <si>
+    <t>OD-02</t>
+  </si>
+  <si>
+    <t>April 2026 public-rules design deck. Not an approved policy (ING-10, 19.3).</t>
+  </si>
+  <si>
+    <t>SRC-21</t>
+  </si>
+  <si>
+    <t>12 - Custodianship of Library Materials (02.08) (1).pdf</t>
+  </si>
+  <si>
+    <t>2008. Verify applicability and evidence passages.</t>
+  </si>
+  <si>
+    <t>SRC-22</t>
+  </si>
+  <si>
+    <t>12 - Technology Usage Policy (06.06) (1).pdf</t>
+  </si>
+  <si>
+    <t>HR12, issued October 2006; applies to all employees, consultants, contractors, temporaries, vendors. Different document from 'Technology Use' (6.13). Check generic 'Company' wording and system references.</t>
+  </si>
+  <si>
+    <t>SRC-23</t>
+  </si>
+  <si>
+    <t>13 - Crisis Management Policy.pdf</t>
+  </si>
+  <si>
+    <t>2008. Check escalation instructions, numbers, applicability, supersession (SAF-8).</t>
+  </si>
+  <si>
+    <t>SRC-24</t>
+  </si>
+  <si>
+    <t>14 - Progressive Discipline Policy (06.06).pdf</t>
+  </si>
+  <si>
+    <t>Check dates, eligibility, labor agreements, legal and HR authority. No disciplinary decisions (GRD-10).</t>
+  </si>
+  <si>
+    <t>SRC-25</t>
+  </si>
+  <si>
+    <t>15 - Service Rating Manual (07.74).pdf</t>
+  </si>
+  <si>
+    <t>1974 reference. Check current relevance and employee agreement implications.</t>
+  </si>
+  <si>
+    <t>SRC-26</t>
+  </si>
+  <si>
+    <t>25 - Family and Medical Leave Act  (06.06).pdf</t>
+  </si>
+  <si>
+    <t>2006. Check dates, eligibility, legal and HR authority. Never calculate current legal entitlements from it (19.4).</t>
+  </si>
+  <si>
+    <t>SRC-27</t>
+  </si>
+  <si>
+    <t>26 - Social Media Policy (03.22) (1).pdf</t>
+  </si>
+  <si>
+    <t>2022. Review confidentiality and current process.</t>
+  </si>
+  <si>
+    <t>SRC-28</t>
+  </si>
+  <si>
+    <t>Ask_BPL_AI_Policy_Test_Script.docx</t>
+  </si>
+  <si>
+    <t>DOCX</t>
+  </si>
+  <si>
+    <t>Text extracted (Word file)</t>
+  </si>
+  <si>
+    <t>Evaluation material</t>
+  </si>
+  <si>
+    <t>Excluded</t>
+  </si>
+  <si>
+    <t>None (not a policy)</t>
+  </si>
+  <si>
+    <t>The 30-question BPL test script (24 in-scope, 6 boundary). Used for GATE-08; never indexed. Counted separately (19.1).</t>
+  </si>
+  <si>
+    <t>SRC-29</t>
+  </si>
+  <si>
+    <t>Guidelines for Public Behavior Violations.pdf</t>
+  </si>
+  <si>
+    <t>Supporting guidance</t>
+  </si>
+  <si>
+    <t>2025 guidance. Supports, and cannot override, the Public Behavior policy (ING-10).</t>
+  </si>
+  <si>
+    <t>SRC-30</t>
+  </si>
+  <si>
+    <t>Public Behavior in the Library Policy (updated Jan-26).docx</t>
+  </si>
+  <si>
+    <t>Policy (draft indicators)</t>
+  </si>
+  <si>
+    <t>OD-02; OD-01</t>
+  </si>
+  <si>
+    <t>Filename says updated Jan-26; internal text says 'Issued: June 2026 (TBD)'. Resolve before answering public-behavior questions.</t>
+  </si>
+  <si>
+    <t>Measure</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>How it is computed</t>
+  </si>
+  <si>
+    <t>Files received</t>
+  </si>
+  <si>
+    <t>All rows (AC-1, GATE-02)</t>
+  </si>
+  <si>
+    <t>Unique by content</t>
+  </si>
+  <si>
+    <t>SHA-256 compared across all 30 files on 2026-10-10; no duplicate content (entered as =B2 because that check was run outside the workbook)</t>
+  </si>
+  <si>
+    <t>BPL documents (excluding test script)</t>
+  </si>
+  <si>
+    <t>Policies, procedures, guidance and deck</t>
+  </si>
+  <si>
+    <t>Eligible (BPL-confirmed current)</t>
+  </si>
+  <si>
+    <t>Zero until BPL confirms authority (OD-01)</t>
+  </si>
+  <si>
+    <t>Includes the extraction-blocked file</t>
+  </si>
+  <si>
+    <t>Extraction blocked (parse check failed)</t>
+  </si>
+  <si>
+    <t>ING-3</t>
+  </si>
+  <si>
+    <t>Excluded from corpus</t>
+  </si>
+  <si>
+    <t>Evaluation script</t>
+  </si>
+  <si>
+    <t>Currently in the pilot index (not confirmed eligible)</t>
+  </si>
+  <si>
+    <t>Byte-identical to the supplied copies; authority still unconfirmed</t>
+  </si>
+  <si>
+    <t>Indexed AND eligible</t>
+  </si>
+  <si>
+    <t>Cannot be claimed yet</t>
+  </si>
+  <si>
+    <t>Documents with a named open decision (OD-02/03/13)</t>
+  </si>
+  <si>
+    <t>Public behavior, emergency/crisis, technology pair</t>
+  </si>
+  <si>
+    <t>Legend: yellow cells on 'Source Inventory' (Owner, Policy number/dates, Reviewer/date) are for Bath Bilissalou / BPL to fill. Every status above is a team disposition, not BPL approval. Parse check only proves text exists; content validation (GATE-04) is still to do.</t>
+  </si>
+  <si>
+    <t>Validated by manual review (Lee Aulder, 2026-10-14</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -486,40 +496,27 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -555,14 +552,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -578,130 +575,42 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8CBAD"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -760,51 +669,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -812,12 +733,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -846,7 +767,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -867,7 +788,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -918,7 +839,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -936,39 +857,38 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N31"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="70" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:14" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1012,7 +932,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -1022,10 +942,10 @@
       <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="3">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="3">
         <v>1886</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -1050,7 +970,7 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
     </row>
-    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>23</v>
       </c>
@@ -1060,10 +980,10 @@
       <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="3">
         <v>2453</v>
       </c>
       <c r="F3" s="3" t="s">
@@ -1088,7 +1008,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
     </row>
-    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
@@ -1098,10 +1018,10 @@
       <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="3">
         <v>4</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="3">
         <v>1967</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1126,7 +1046,7 @@
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>34</v>
       </c>
@@ -1136,10 +1056,10 @@
       <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="3">
         <v>2</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="3">
         <v>2434</v>
       </c>
       <c r="F5" s="3" t="s">
@@ -1164,7 +1084,7 @@
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
@@ -1174,10 +1094,10 @@
       <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="3">
         <v>5</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="3">
         <v>2205</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -1202,7 +1122,7 @@
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>40</v>
       </c>
@@ -1212,10 +1132,10 @@
       <c r="C7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="3">
         <v>4</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="3">
         <v>2172</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -1240,7 +1160,7 @@
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>43</v>
       </c>
@@ -1250,10 +1170,10 @@
       <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="3">
         <v>2</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="3">
         <v>1286</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -1278,7 +1198,7 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>46</v>
       </c>
@@ -1288,10 +1208,10 @@
       <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="3">
         <v>7</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="3">
         <v>2045</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -1316,7 +1236,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
@@ -1326,10 +1246,10 @@
       <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="3">
         <v>8</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="3">
         <v>1512</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -1354,7 +1274,7 @@
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>52</v>
       </c>
@@ -1364,10 +1284,10 @@
       <c r="C11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="3">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="3">
         <v>1845</v>
       </c>
       <c r="F11" s="3" t="s">
@@ -1392,7 +1312,7 @@
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>55</v>
       </c>
@@ -1402,10 +1322,10 @@
       <c r="C12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="3">
         <v>6</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="3">
         <v>1579</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -1430,7 +1350,7 @@
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
     </row>
-    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>58</v>
       </c>
@@ -1440,10 +1360,10 @@
       <c r="C13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="3">
         <v>7</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="3">
         <v>2299</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -1468,7 +1388,7 @@
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>61</v>
       </c>
@@ -1478,14 +1398,14 @@
       <c r="C14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="3">
         <v>10</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="3">
         <v>248</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>63</v>
+      <c r="F14" s="9" t="s">
+        <v>146</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>30</v>
@@ -1493,33 +1413,33 @@
       <c r="H14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="3">
         <v>4</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="3">
         <v>2132</v>
       </c>
       <c r="F15" s="3" t="s">
@@ -1538,26 +1458,26 @@
         <v>26</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="3">
         <v>3</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="3">
         <v>2085</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -1582,20 +1502,20 @@
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="3">
         <v>11</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="3">
         <v>2811</v>
       </c>
       <c r="F17" s="3" t="s">
@@ -1614,26 +1534,26 @@
         <v>26</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
     </row>
-    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="3">
         <v>2</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="3">
         <v>2046</v>
       </c>
       <c r="F18" s="3" t="s">
@@ -1658,20 +1578,20 @@
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
     </row>
-    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="3">
         <v>3</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="3">
         <v>2454</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -1696,20 +1616,20 @@
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
     </row>
-    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="3">
         <v>2</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="3">
         <v>1714</v>
       </c>
       <c r="F20" s="3" t="s">
@@ -1728,26 +1648,26 @@
         <v>26</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
     </row>
-    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="3">
         <v>11</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="3">
         <v>1645</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -1757,35 +1677,35 @@
         <v>18</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="K21" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
     </row>
-    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="3">
         <v>2</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="3">
         <v>1904</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -1804,26 +1724,26 @@
         <v>26</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
     </row>
-    <row r="23" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="3">
         <v>5</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="3">
         <v>2333</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -1842,26 +1762,26 @@
         <v>32</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="3">
         <v>7</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="3">
         <v>1606</v>
       </c>
       <c r="F24" s="3" t="s">
@@ -1880,26 +1800,26 @@
         <v>21</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
     </row>
-    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="3">
         <v>3</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="3">
         <v>2854</v>
       </c>
       <c r="F25" s="3" t="s">
@@ -1918,26 +1838,26 @@
         <v>26</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
       <c r="N25" s="4"/>
     </row>
-    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="3">
         <v>9</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="3">
         <v>1943</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1956,26 +1876,26 @@
         <v>26</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
     </row>
-    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="3">
         <v>4</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="3">
         <v>2905</v>
       </c>
       <c r="F27" s="3" t="s">
@@ -1994,26 +1914,26 @@
         <v>26</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="3">
         <v>6</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="3">
         <v>4797</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -2032,60 +1952,60 @@
         <v>26</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
     </row>
-    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>18</v>
       </c>
       <c r="H29" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="J29" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="K29" s="3" t="s">
         <v>113</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
     </row>
-    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="3">
         <v>7</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="3">
         <v>2425</v>
       </c>
       <c r="F30" s="3" t="s">
@@ -2095,229 +2015,215 @@
         <v>18</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>20</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="L30" s="4"/>
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
     </row>
-    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>18</v>
       </c>
       <c r="H31" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="K31" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="K31" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
       <c r="N31" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N31"/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <autoFilter ref="A1:N31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="80"/>
+    <col min="1" max="1" width="52" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="7" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="B2" s="7">
+        <f>COUNTA('Source Inventory'!A2:A31)</f>
+        <v>30</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="8" t="n">
-        <f aca="false">COUNTA('Source Inventory'!A2:A31)</f>
+      <c r="B3" s="7">
+        <f>B2</f>
         <v>30</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="8" t="n">
-        <f aca="false">B2</f>
-        <v>30</v>
-      </c>
-      <c r="C3" s="8" t="s">
+      <c r="B4" s="7">
+        <f>B2-COUNTIF('Source Inventory'!H2:H31,"Evaluation material")</f>
+        <v>29</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <f aca="false">B2-COUNTIF('Source Inventory'!H2:H31,"Evaluation material")</f>
+      <c r="B5" s="7">
+        <f>COUNTIF('Source Inventory'!I2:I31,"Eligible*")</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="7">
+        <f>COUNTIF('Source Inventory'!I2:I31,"Authority pending*")</f>
         <v>29</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <f aca="false">COUNTIF('Source Inventory'!I2:I31,"Eligible*")</f>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="7">
+        <f>COUNTIF('Source Inventory'!F2:F31,"FAIL*")</f>
         <v>0</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="8" t="n">
-        <f aca="false">COUNTIF('Source Inventory'!I2:I31,"Authority pending*")</f>
-        <v>29</v>
-      </c>
-      <c r="C6" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <f aca="false">COUNTIF('Source Inventory'!F2:F31,"FAIL*")</f>
+      <c r="B8" s="7">
+        <f>COUNTIF('Source Inventory'!I2:I31,"Excluded")</f>
         <v>1</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <f aca="false">COUNTIF('Source Inventory'!I2:I31,"Excluded")</f>
-        <v>1</v>
-      </c>
-      <c r="C8" s="8" t="s">
+      <c r="B9" s="7">
+        <f>COUNTIF('Source Inventory'!G2:G31,"Yes")</f>
+        <v>8</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <f aca="false">COUNTIF('Source Inventory'!G2:G31,"Yes")</f>
+      <c r="B10" s="7">
+        <f>COUNTIFS('Source Inventory'!G2:G31,"Yes",'Source Inventory'!I2:I31,"Eligible*")</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="7">
+        <f>SUMPRODUCT(--(ISNUMBER(SEARCH("OD-0",'Source Inventory'!J2:J31))),--(ISNUMBER(SEARCH("OD-02",'Source Inventory'!J2:J31))+ISNUMBER(SEARCH("OD-03",'Source Inventory'!J2:J31))+ISNUMBER(SEARCH("OD-13",'Source Inventory'!J2:J31))&gt;0))</f>
         <v>8</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B10" s="8" t="n">
-        <f aca="false">COUNTIFS('Source Inventory'!G2:G31,"Yes",'Source Inventory'!I2:I31,"Eligible*")</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+    <row r="14" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <f aca="false">SUMPRODUCT(--(ISNUMBER(SEARCH("OD-0",'Source Inventory'!J2:J31))),--(ISNUMBER(SEARCH("OD-02",'Source Inventory'!J2:J31))+ISNUMBER(SEARCH("OD-03",'Source Inventory'!J2:J31))+ISNUMBER(SEARCH("OD-13",'Source Inventory'!J2:J31))&gt;0))</f>
-        <v>8</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A14:C14"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>